<commit_message>
varaint and image foler fixes
</commit_message>
<xml_diff>
--- a/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -390,7 +390,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ6"/>
+  <dimension ref="A1:BE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,6 +428,31 @@
           <t>Terracota Style With Plant and Gym equipment in background</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Glacier Veil Studio</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Arctic Linen Studio</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Moonstone Plane Studio</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Porcelain Arc Studio</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Opal Grid Studio</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -540,6 +565,11 @@
           <t>Graphite Pearl Studio</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Opaline Panel Studio</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -762,6 +792,111 @@
       <c r="AJ6" t="inlineStr">
         <is>
           <t>Opal Mist Studio</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>Talc Panel Studio</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Halo Composite Studio</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>Moonwash Composite Studio</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Siltstone Horizon Studio</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Ivory Basalt Studio</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Dune Paper Studio</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Calcium Arc Studio</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>Gypsum Fold Studio</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>Velum Stone Studio</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Ecru Monolith Studio</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Ivory Relief Studio</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>Putty Wave Studio</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>Sage Mist Panel Studio</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>Vanilla Seam Studio</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>Sesame Horizon Studio</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>Driftstone Layer Studio</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Cashstone Inlay Studio</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Dolomite Frame Studio</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>Marshmallow Edge Studio</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>Graphite Ribbon Studio</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>Nimbus Groove Studio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed Crash Bug on Order-Sorter
</commit_message>
<xml_diff>
--- a/image_prompter/USED-IMAGE-DESIGNS.xlsx
+++ b/image_prompter/USED-IMAGE-DESIGNS.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4d750000efd74353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R827ed1a23e554bc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -703,6 +703,36 @@
       <x:c r="AI4" t="str">
         <x:v>Cranberry Quartz-Flax Studio</x:v>
       </x:c>
+      <x:c r="AJ4" t="str">
+        <x:v>Pearl Sand Fine-Rake Plaster Studio</x:v>
+      </x:c>
+      <x:c r="AK4" t="str">
+        <x:v>Pale Apricot Mineral-Wash Studio</x:v>
+      </x:c>
+      <x:c r="AL4" t="str">
+        <x:v>Light Celadon Basket-Weave Render Studio</x:v>
+      </x:c>
+      <x:c r="AM4" t="str">
+        <x:v>Warm Ivory Split-Face Limestone Studio</x:v>
+      </x:c>
+      <x:c r="AN4" t="str">
+        <x:v>Mist Lavender Silk-Gesso Studio</x:v>
+      </x:c>
+      <x:c r="AO4" t="str">
+        <x:v>Powder Blue Micro-Fluted Clay Studio</x:v>
+      </x:c>
+      <x:c r="AP4" t="str">
+        <x:v>Soft Oat Travertine-Pore Studio</x:v>
+      </x:c>
+      <x:c r="AQ4" t="str">
+        <x:v>Blush Beige Cross-Trowel Studio</x:v>
+      </x:c>
+      <x:c r="AR4" t="str">
+        <x:v>Pale Buttercream Woven-Lime Studio</x:v>
+      </x:c>
+      <x:c r="AS4" t="str">
+        <x:v>Frost Mint Porcelain-Grain Studio</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="inlineStr">

</xml_diff>